<commit_message>
Daily slate 2026-06-06 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-06-04.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-06-04.xlsx
@@ -471,16 +471,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>134</v>
+        <v>20</v>
       </c>
       <c r="E2" t="n">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="F2" t="n">
-        <v>69</v>
+        <v>9</v>
       </c>
       <c r="G2" t="n">
-        <v>48.5</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3">
@@ -500,16 +500,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>191</v>
+        <v>181</v>
       </c>
       <c r="E3" t="n">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="F3" t="n">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="G3" t="n">
-        <v>53.9</v>
+        <v>55.8</v>
       </c>
     </row>
     <row r="4">
@@ -529,16 +529,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="E4" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F4" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="G4" t="n">
-        <v>54.8</v>
+        <v>54.7</v>
       </c>
     </row>
     <row r="5">
@@ -587,16 +587,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>60</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>325</v>
+        <v>444</v>
       </c>
       <c r="E8" t="n">
-        <v>106</v>
+        <v>162</v>
       </c>
       <c r="F8" t="n">
-        <v>219</v>
+        <v>282</v>
       </c>
       <c r="G8" t="n">
-        <v>32.6</v>
+        <v>36.5</v>
       </c>
     </row>
     <row r="9">
@@ -671,16 +671,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="E9" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="F9" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="G9" t="n">
-        <v>62.5</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10">
@@ -729,16 +729,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>650</v>
+        <v>675</v>
       </c>
       <c r="E11" t="n">
-        <v>409</v>
+        <v>421</v>
       </c>
       <c r="F11" t="n">
-        <v>241</v>
+        <v>254</v>
       </c>
       <c r="G11" t="n">
-        <v>62.9</v>
+        <v>62.4</v>
       </c>
     </row>
     <row r="12">
@@ -758,16 +758,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E12" t="n">
         <v>85</v>
       </c>
       <c r="F12" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G12" t="n">
-        <v>72.59999999999999</v>
+        <v>72</v>
       </c>
     </row>
     <row r="13">
@@ -816,16 +816,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>204</v>
+        <v>213</v>
       </c>
       <c r="E14" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F14" t="n">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="G14" t="n">
-        <v>26.5</v>
+        <v>25.8</v>
       </c>
     </row>
     <row r="15">
@@ -845,16 +845,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>282</v>
+        <v>291</v>
       </c>
       <c r="E15" t="n">
         <v>54</v>
       </c>
       <c r="F15" t="n">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="G15" t="n">
-        <v>19.1</v>
+        <v>18.6</v>
       </c>
     </row>
     <row r="16">
@@ -903,16 +903,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>2677</v>
+        <v>2794</v>
       </c>
       <c r="E17" t="n">
-        <v>569</v>
+        <v>588</v>
       </c>
       <c r="F17" t="n">
-        <v>2108</v>
+        <v>2206</v>
       </c>
       <c r="G17" t="n">
-        <v>21.3</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -1151,34 +1151,28 @@
         <v>31</v>
       </c>
       <c r="R2" t="n">
-        <v>48.4</v>
+        <v>58.3</v>
       </c>
       <c r="S2" t="n">
-        <v>126</v>
-      </c>
-      <c r="T2" t="n">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="U2" t="n">
-        <v>2</v>
-      </c>
-      <c r="V2" t="n">
-        <v>33.3</v>
+        <v>0</v>
       </c>
       <c r="W2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="X2" t="n">
-        <v>32.5</v>
+        <v>37.2</v>
       </c>
       <c r="Y2" t="n">
-        <v>249</v>
+        <v>368</v>
       </c>
       <c r="Z2" t="n">
-        <v>50</v>
+        <v>52.9</v>
       </c>
       <c r="AA2" t="n">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="AB2" t="n">
         <v>33.3</v>
@@ -1189,8 +1183,11 @@
       <c r="AE2" t="n">
         <v>0</v>
       </c>
+      <c r="AF2" t="n">
+        <v>42.9</v>
+      </c>
       <c r="AG2" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3">
@@ -1492,16 +1489,16 @@
         <v>87</v>
       </c>
       <c r="D7" t="n">
-        <v>62.9</v>
+        <v>62.4</v>
       </c>
       <c r="E7" t="n">
-        <v>650</v>
+        <v>675</v>
       </c>
       <c r="F7" t="n">
-        <v>72.59999999999999</v>
+        <v>72</v>
       </c>
       <c r="G7" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="H7" t="n">
         <v>37.7</v>
@@ -1510,16 +1507,16 @@
         <v>122</v>
       </c>
       <c r="J7" t="n">
-        <v>26.5</v>
+        <v>25.8</v>
       </c>
       <c r="K7" t="n">
-        <v>204</v>
+        <v>213</v>
       </c>
       <c r="L7" t="n">
-        <v>19.1</v>
+        <v>18.6</v>
       </c>
       <c r="M7" t="n">
-        <v>282</v>
+        <v>291</v>
       </c>
       <c r="N7" t="n">
         <v>12</v>
@@ -1528,40 +1525,40 @@
         <v>158</v>
       </c>
       <c r="P7" t="n">
-        <v>21.3</v>
+        <v>21</v>
       </c>
       <c r="Q7" t="n">
-        <v>2677</v>
+        <v>2794</v>
       </c>
       <c r="R7" t="n">
-        <v>48.5</v>
+        <v>55</v>
       </c>
       <c r="S7" t="n">
-        <v>134</v>
+        <v>20</v>
       </c>
       <c r="T7" t="n">
-        <v>54.8</v>
+        <v>54.7</v>
       </c>
       <c r="U7" t="n">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="V7" t="n">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="W7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="X7" t="n">
-        <v>32.6</v>
+        <v>36.5</v>
       </c>
       <c r="Y7" t="n">
-        <v>325</v>
+        <v>444</v>
       </c>
       <c r="Z7" t="n">
-        <v>53.9</v>
+        <v>55.8</v>
       </c>
       <c r="AA7" t="n">
-        <v>191</v>
+        <v>181</v>
       </c>
       <c r="AB7" t="n">
         <v>46.2</v>
@@ -1573,10 +1570,10 @@
         <v>0</v>
       </c>
       <c r="AF7" t="n">
-        <v>62.5</v>
+        <v>50</v>
       </c>
       <c r="AG7" t="n">
-        <v>8</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>